<commit_message>
Changed power supply. Added THT to SMD Assembly. Regenerated Project Outputs
</commit_message>
<xml_diff>
--- a/Project Outputs for UZ_A_MAX11331_Daugther/BOM/BOM_UZ_A_MAX11331_Daugther_2v01.xlsx
+++ b/Project Outputs for UZ_A_MAX11331_Daugther/BOM/BOM_UZ_A_MAX11331_Daugther_2v01.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\UltraZohm\UZ_A_MAX11331_Daughter\Project Outputs for UZ_A_MAX11331_Daugther\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thoma\Documents\Altium\UltraZOhm\UZ_A_MAX11331_Daughter\Project Outputs for UZ_A_MAX11331_Daugther\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6EA26938-FAD7-414E-9FE9-A4DA64B3F0B0}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B067676D-2180-47B7-9D6C-448ADF7F9E56}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2940" yWindow="2460" windowWidth="14670" windowHeight="8325" xr2:uid="{F41EB0CD-8ED5-4C14-B542-4E32C508796F}"/>
+    <workbookView xWindow="1500" yWindow="180" windowWidth="21600" windowHeight="11385" xr2:uid="{BF8BCF2F-7E93-4DE2-A197-B1E70D134EA6}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM_UZ_A_MAX11331_Daugther_2v01" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="421" uniqueCount="224">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="216">
   <si>
     <t>Name</t>
   </si>
@@ -195,7 +195,7 @@
     <t>399-8140-1-ND</t>
   </si>
   <si>
-    <t>C14A, C14B, C14C, C14D, C14E, C14F, C14G, C14H, C15A, C15B, C15C, C15D, C15E, C15F, C15G, C15H, C16A, C16B, C16C, C16D, C16E, C16F, C16G, C16H, C17A, C17B, C17C, C17D, C17E, C17F, C17G, C17H, C22A, C22B, C22C, C22D, C22E, C22F, C22G, C22H, C23A, C23B, C23C, C23D, C23E, C23F, C23G, C23H, C24A, C24B, C24C, C24D, C24E, C24F, C24G, C24H, C25A, C25B, C25C, C25D, C25E, C25F, C25G, C25H, C27A, C27B, C27C, C27D, C28A, C28B, C28C, C28D, C30A, C30B, C30C, C30D, C34A, C34B, C34C, C34D, C35, C36, C37, C38, C39, C40, C45, C48</t>
+    <t>C14A, C14B, C14C, C14D, C14E, C14F, C14G, C14H, C15A, C15B, C15C, C15D, C15E, C15F, C15G, C15H, C16A, C16B, C16C, C16D, C16E, C16F, C16G, C16H, C17A, C17B, C17C, C17D, C17E, C17F, C17G, C17H, C22A, C22B, C22C, C22D, C22E, C22F, C22G, C22H, C23A, C23B, C23C, C23D, C23E, C23F, C23G, C23H, C24A, C24B, C24C, C24D, C24E, C24F, C24G, C24H, C25A, C25B, C25C, C25D, C25E, C25F, C25G, C25H, C27A, C27B, C27C, C27D, C28A, C28B, C28C, C28D, C30A, C30B, C30C, C30D, C34A, C34B, C34C, C34D, C35, C36, C38, C39, C40, C41, C45, C48</t>
   </si>
   <si>
     <t>C0603C104M5RACTU</t>
@@ -225,13 +225,16 @@
     <t>Capacitor Ceramic</t>
   </si>
   <si>
+    <t>Digikey</t>
+  </si>
+  <si>
     <t>587-5869-1-ND</t>
   </si>
   <si>
     <t>1µF</t>
   </si>
   <si>
-    <t>C29</t>
+    <t>C29, C42</t>
   </si>
   <si>
     <t>C0603C105K3RACTU</t>
@@ -258,28 +261,22 @@
     <t>732-7925-1-ND</t>
   </si>
   <si>
-    <t>2.2nF</t>
-  </si>
-  <si>
-    <t>C41</t>
-  </si>
-  <si>
-    <t>C0603C222K5RAC7411</t>
-  </si>
-  <si>
-    <t>399-17586-1-ND</t>
-  </si>
-  <si>
-    <t>1.2nF</t>
-  </si>
-  <si>
-    <t>C42</t>
-  </si>
-  <si>
-    <t>C0603C122K5RACTU</t>
-  </si>
-  <si>
-    <t>399-7851-1-ND</t>
+    <t>68µF</t>
+  </si>
+  <si>
+    <t>C43, C44</t>
+  </si>
+  <si>
+    <t>+/-20%</t>
+  </si>
+  <si>
+    <t>WCAP-ATG8 THT Aluminum Electrolytic Capacitors, D6.3mm x L11mm, 68uF, +/-20%, 35VDC</t>
+  </si>
+  <si>
+    <t>WCAP-ATG8_6.3x11</t>
+  </si>
+  <si>
+    <t>732-8736-1-ND</t>
   </si>
   <si>
     <t>10µF</t>
@@ -300,21 +297,6 @@
     <t>490-9964-1-ND</t>
   </si>
   <si>
-    <t>91pF</t>
-  </si>
-  <si>
-    <t>C50</t>
-  </si>
-  <si>
-    <t>Murata</t>
-  </si>
-  <si>
-    <t>GRM1885C1H910JA01D</t>
-  </si>
-  <si>
-    <t>490-1426-1-ND</t>
-  </si>
-  <si>
     <t>Bright Green, 2V</t>
   </si>
   <si>
@@ -351,25 +333,37 @@
     <t>732-4966-1-ND</t>
   </si>
   <si>
-    <t>33µH</t>
+    <t>Conector RJ-45 4x2</t>
+  </si>
+  <si>
+    <t>J1</t>
+  </si>
+  <si>
+    <t>TE Connectivity</t>
+  </si>
+  <si>
+    <t>1-1734715-2</t>
+  </si>
+  <si>
+    <t>RJ45 - 4x2</t>
+  </si>
+  <si>
+    <t>A118195-ND</t>
+  </si>
+  <si>
+    <t>15mH</t>
   </si>
   <si>
     <t>L1</t>
   </si>
   <si>
-    <t>Taiyo Yuden</t>
-  </si>
-  <si>
-    <t>NRS5030T330MMGJ</t>
-  </si>
-  <si>
-    <t>SMT power Inductor, 33µH, 225m DRC</t>
-  </si>
-  <si>
-    <t>Inductor 5030</t>
-  </si>
-  <si>
-    <t>587-3458-1-ND</t>
+    <t>SMT power Inductor, 15uH, 40m DRC</t>
+  </si>
+  <si>
+    <t>SMT_inductor_1050_Performance</t>
+  </si>
+  <si>
+    <t>811-3837-1-ND</t>
   </si>
   <si>
     <t>1M</t>
@@ -462,15 +456,6 @@
     <t>311-160FRCT-ND</t>
   </si>
   <si>
-    <t>0</t>
-  </si>
-  <si>
-    <t>R24</t>
-  </si>
-  <si>
-    <t>311-0.0GRCT-ND</t>
-  </si>
-  <si>
     <t>100R</t>
   </si>
   <si>
@@ -483,7 +468,7 @@
     <t>311-100HRCT-ND</t>
   </si>
   <si>
-    <t>R28, R29, R30, R34</t>
+    <t>R28, R29, R30</t>
   </si>
   <si>
     <t>RC0603FR-0710KL</t>
@@ -504,40 +489,25 @@
     <t>YAG3329CT-ND</t>
   </si>
   <si>
-    <t>200k</t>
+    <t>100k</t>
   </si>
   <si>
     <t>R32</t>
   </si>
   <si>
-    <t>RC0603FR-07200KL</t>
-  </si>
-  <si>
-    <t>311-200KHRCT-ND</t>
-  </si>
-  <si>
-    <t>115k</t>
+    <t>RC0603FR-07100KL</t>
+  </si>
+  <si>
+    <t>311-100KHRCT-ND</t>
+  </si>
+  <si>
+    <t>38.3k</t>
   </si>
   <si>
     <t>R33</t>
   </si>
   <si>
-    <t>RC0603FR-07115KL</t>
-  </si>
-  <si>
-    <t>311-115KHRCT-ND</t>
-  </si>
-  <si>
-    <t>100k</t>
-  </si>
-  <si>
-    <t>R35</t>
-  </si>
-  <si>
-    <t>RC0603FR-07100KL</t>
-  </si>
-  <si>
-    <t>311-100KHRCT-ND</t>
+    <t>311-38.3KHRCT-ND</t>
   </si>
   <si>
     <t>220</t>
@@ -672,43 +642,49 @@
     <t>ADN4665ARUZ-ND</t>
   </si>
   <si>
-    <t>Single LVDS driver</t>
-  </si>
-  <si>
-    <t>U8</t>
-  </si>
-  <si>
-    <t>ADN4661BRZ</t>
-  </si>
-  <si>
-    <t>Single, 3V, CMOS, LVDS High Speed differential driver</t>
-  </si>
-  <si>
-    <t>SOIC127P600X170_HS-9N_no_THP</t>
-  </si>
-  <si>
-    <t>ADN4661BRZ-ND</t>
-  </si>
-  <si>
-    <t>buck converter</t>
+    <t>Buck Converter</t>
   </si>
   <si>
     <t>U9</t>
   </si>
   <si>
-    <t>LM5163DDAR</t>
-  </si>
-  <si>
-    <t>100V Input, 0.5A Synchronous Buck DC/DC Converter with Ultra-low Iq</t>
+    <t>3.8V to 36V, 2A synchronous step-down converter</t>
   </si>
   <si>
     <t>SOIC127P600X170_HS-9N</t>
   </si>
   <si>
-    <t>Digikey</t>
-  </si>
-  <si>
-    <t>296-LM5163HQDDARQ1CT-ND</t>
+    <t>296-48841-ND</t>
+  </si>
+  <si>
+    <t>IPL1-102-01-L-D-K</t>
+  </si>
+  <si>
+    <t>X1</t>
+  </si>
+  <si>
+    <t>Samtec</t>
+  </si>
+  <si>
+    <t>2.54mm Double Row Terminal Assembly, Right-Angled</t>
+  </si>
+  <si>
+    <t>SAM10565-ND</t>
+  </si>
+  <si>
+    <t>2x8 Pin</t>
+  </si>
+  <si>
+    <t>X2</t>
+  </si>
+  <si>
+    <t>EHF-108-01-F-D</t>
+  </si>
+  <si>
+    <t>Dual Row, 2x8 Shrouded IDC Header with Ejectors 50 mil pitch</t>
+  </si>
+  <si>
+    <t>SAM9265-ND</t>
   </si>
 </sst>
 </file>
@@ -779,7 +755,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -795,7 +771,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -1090,24 +1066,24 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{455B81CA-AC47-43B9-A7FD-1B0D85DF59C0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C211915-C694-414D-8EA1-5E284EE500B0}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P39"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:P37"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.5703125" customWidth="1"/>
-    <col min="2" max="2" width="17.42578125" customWidth="1"/>
-    <col min="3" max="3" width="18.7109375" customWidth="1"/>
-    <col min="4" max="4" width="21" customWidth="1"/>
-    <col min="5" max="5" width="16.5703125" customWidth="1"/>
-    <col min="6" max="6" width="13.7109375" customWidth="1"/>
-    <col min="7" max="9" width="16.5703125" customWidth="1"/>
-    <col min="10" max="11" width="12.7109375" customWidth="1"/>
-    <col min="12" max="12" width="12.28515625" customWidth="1"/>
-    <col min="13" max="13" width="15.5703125" customWidth="1"/>
-    <col min="14" max="16" width="16.5703125" customWidth="1"/>
+    <col min="1" max="1" width="18.85546875" customWidth="1"/>
+    <col min="2" max="2" width="17.7109375" customWidth="1"/>
+    <col min="3" max="3" width="19" customWidth="1"/>
+    <col min="4" max="4" width="21.28515625" customWidth="1"/>
+    <col min="5" max="5" width="16.7109375" customWidth="1"/>
+    <col min="6" max="6" width="13.85546875" customWidth="1"/>
+    <col min="7" max="9" width="16.7109375" customWidth="1"/>
+    <col min="10" max="11" width="12.85546875" customWidth="1"/>
+    <col min="12" max="12" width="12.42578125" customWidth="1"/>
+    <col min="13" max="13" width="15.85546875" customWidth="1"/>
+    <col min="14" max="16" width="16.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" s="1" customFormat="1" ht="30" x14ac:dyDescent="0.25">
@@ -1252,7 +1228,7 @@
         <v>0.17</v>
       </c>
     </row>
-    <row r="4" spans="1:16" ht="330" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:16" ht="315" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>33</v>
       </c>
@@ -1487,45 +1463,41 @@
         <v>41</v>
       </c>
       <c r="L8" s="3" t="s">
-        <v>23</v>
+        <v>62</v>
       </c>
       <c r="M8" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="N8" s="4">
-        <v>8.6999999999999994E-2</v>
-      </c>
+        <v>63</v>
+      </c>
+      <c r="N8" s="4"/>
       <c r="O8" s="4">
         <v>8</v>
       </c>
-      <c r="P8" s="4">
-        <v>0.87</v>
-      </c>
+      <c r="P8" s="4"/>
     </row>
     <row r="9" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C9" s="3" t="s">
         <v>49</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>37</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="G9" s="3" t="s">
         <v>28</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I9" s="3" t="s">
         <v>30</v>
@@ -1540,42 +1512,42 @@
         <v>23</v>
       </c>
       <c r="M9" s="3" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="N9" s="4">
         <v>0.28000000000000003</v>
       </c>
       <c r="O9" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P9" s="4">
-        <v>0.28000000000000003</v>
+        <v>0.56000000000000005</v>
       </c>
     </row>
     <row r="10" spans="1:16" ht="45" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C10" s="3" t="s">
         <v>18</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>37</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="G10" s="3" t="s">
         <v>28</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="I10" s="3" t="s">
         <v>30</v>
@@ -1590,7 +1562,7 @@
         <v>23</v>
       </c>
       <c r="M10" s="3" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="N10" s="4">
         <v>2.1000000000000001E-2</v>
@@ -1602,727 +1574,701 @@
         <v>0.21</v>
       </c>
     </row>
-    <row r="11" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:16" ht="135" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B11" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="C11" s="4"/>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4"/>
+      <c r="F11" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="C11" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>73</v>
-      </c>
       <c r="G11" s="3" t="s">
-        <v>28</v>
+        <v>76</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="I11" s="3" t="s">
-        <v>30</v>
-      </c>
+        <v>54</v>
+      </c>
+      <c r="I11" s="4"/>
       <c r="J11" s="3" t="s">
-        <v>61</v>
+        <v>77</v>
       </c>
       <c r="K11" s="3" t="s">
-        <v>41</v>
+        <v>78</v>
       </c>
       <c r="L11" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M11" s="3" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="N11" s="4">
-        <v>0.1</v>
+        <v>0.13</v>
       </c>
       <c r="O11" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P11" s="4">
-        <v>0.1</v>
+        <v>0.26</v>
       </c>
     </row>
     <row r="12" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>49</v>
+        <v>82</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="E12" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="I12" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="J12" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="K12" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="L12" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="M12" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="N12" s="4">
+        <v>0.34</v>
+      </c>
+      <c r="O12" s="4">
+        <v>2</v>
+      </c>
+      <c r="P12" s="4">
+        <v>0.68</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" ht="120" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="E13" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="F12" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="G12" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="H12" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="I12" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="J12" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="K12" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="L12" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="M12" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="N12" s="4">
-        <v>0.1</v>
-      </c>
-      <c r="O12" s="4">
+      <c r="F13" s="4"/>
+      <c r="G13" s="4"/>
+      <c r="H13" s="4"/>
+      <c r="I13" s="4"/>
+      <c r="J13" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="K13" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="L13" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="M13" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="N13" s="4">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="O13" s="4">
         <v>1</v>
       </c>
-      <c r="P12" s="4">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:16" ht="30" x14ac:dyDescent="0.25">
-      <c r="A13" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="D13" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="E13" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="F13" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="G13" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="H13" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="I13" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="J13" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="K13" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="L13" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="M13" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="N13" s="4">
-        <v>0.34</v>
-      </c>
-      <c r="O13" s="4">
-        <v>2</v>
-      </c>
       <c r="P13" s="4">
-        <v>0.68</v>
-      </c>
-    </row>
-    <row r="14" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+        <v>0.14000000000000001</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" ht="120" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="B14" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="C14" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="C14" s="3" t="s">
-        <v>89</v>
-      </c>
       <c r="D14" s="3" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="E14" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="F14" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="G14" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="H14" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="I14" s="3" t="s">
-        <v>40</v>
-      </c>
+      <c r="F14" s="4"/>
+      <c r="G14" s="4"/>
+      <c r="H14" s="4"/>
+      <c r="I14" s="4"/>
       <c r="J14" s="3" t="s">
-        <v>61</v>
+        <v>96</v>
       </c>
       <c r="K14" s="3" t="s">
-        <v>41</v>
+        <v>91</v>
       </c>
       <c r="L14" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M14" s="3" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="N14" s="4">
-        <v>0.12</v>
+        <v>0.16</v>
       </c>
       <c r="O14" s="4">
         <v>1</v>
       </c>
       <c r="P14" s="4">
-        <v>0.12</v>
-      </c>
-    </row>
-    <row r="15" spans="1:16" ht="120" x14ac:dyDescent="0.25">
+        <v>0.16</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="E15" s="3" t="s">
-        <v>37</v>
-      </c>
+        <v>101</v>
+      </c>
+      <c r="E15" s="4"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
       <c r="I15" s="4"/>
       <c r="J15" s="3" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="K15" s="3" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="L15" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M15" s="3" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="N15" s="4">
-        <v>0.14000000000000001</v>
+        <v>13.37</v>
       </c>
       <c r="O15" s="4">
         <v>1</v>
       </c>
       <c r="P15" s="4">
-        <v>0.14000000000000001</v>
-      </c>
-    </row>
-    <row r="16" spans="1:16" ht="120" x14ac:dyDescent="0.25">
+        <v>13.37</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" ht="60" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="C16" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="D16" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="E16" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="F16" s="4"/>
+        <v>105</v>
+      </c>
+      <c r="C16" s="4"/>
+      <c r="D16" s="4"/>
+      <c r="E16" s="4"/>
+      <c r="F16" s="3" t="s">
+        <v>104</v>
+      </c>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
       <c r="I16" s="4"/>
       <c r="J16" s="3" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="K16" s="3" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="L16" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M16" s="3" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="N16" s="4">
-        <v>0.16</v>
+        <v>1.36</v>
       </c>
       <c r="O16" s="4">
         <v>1</v>
       </c>
       <c r="P16" s="4">
-        <v>0.16</v>
-      </c>
-    </row>
-    <row r="17" spans="1:16" ht="60" x14ac:dyDescent="0.25">
+        <v>1.36</v>
+      </c>
+    </row>
+    <row r="17" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="E17" s="4"/>
+        <v>112</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>20</v>
+      </c>
       <c r="F17" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="G17" s="4"/>
+        <v>109</v>
+      </c>
+      <c r="G17" s="3" t="s">
+        <v>113</v>
+      </c>
       <c r="H17" s="4"/>
       <c r="I17" s="4"/>
       <c r="J17" s="3" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="K17" s="3" t="s">
-        <v>109</v>
+        <v>22</v>
       </c>
       <c r="L17" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M17" s="3" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="N17" s="4">
-        <v>0.33</v>
+        <v>0.1</v>
       </c>
       <c r="O17" s="4">
         <v>1</v>
       </c>
       <c r="P17" s="4">
-        <v>0.33</v>
-      </c>
-    </row>
-    <row r="18" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16" ht="90" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="E18" s="3" t="s">
-        <v>20</v>
-      </c>
+        <v>119</v>
+      </c>
+      <c r="E18" s="4"/>
       <c r="F18" s="3" t="s">
-        <v>111</v>
-      </c>
-      <c r="G18" s="3" t="s">
-        <v>115</v>
-      </c>
+        <v>116</v>
+      </c>
+      <c r="G18" s="4"/>
       <c r="H18" s="4"/>
       <c r="I18" s="4"/>
       <c r="J18" s="3" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="K18" s="3" t="s">
-        <v>22</v>
+        <v>121</v>
       </c>
       <c r="L18" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M18" s="3" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="N18" s="4">
-        <v>0.1</v>
+        <v>0.60299999999999998</v>
       </c>
       <c r="O18" s="4">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="P18" s="4">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="19" spans="1:16" ht="90" x14ac:dyDescent="0.25">
+        <v>9.65</v>
+      </c>
+    </row>
+    <row r="19" spans="1:16" ht="315" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="E19" s="4"/>
+        <v>126</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>37</v>
+      </c>
       <c r="F19" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="G19" s="4"/>
+        <v>123</v>
+      </c>
+      <c r="G19" s="3" t="s">
+        <v>127</v>
+      </c>
       <c r="H19" s="4"/>
       <c r="I19" s="4"/>
       <c r="J19" s="3" t="s">
-        <v>122</v>
+        <v>82</v>
       </c>
       <c r="K19" s="3" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="L19" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M19" s="3" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="N19" s="4">
-        <v>0.60299999999999998</v>
+        <v>0.10150000000000001</v>
       </c>
       <c r="O19" s="4">
-        <v>16</v>
+        <v>64</v>
       </c>
       <c r="P19" s="4">
-        <v>9.65</v>
-      </c>
-    </row>
-    <row r="20" spans="1:16" ht="330" x14ac:dyDescent="0.25">
+        <v>10.15</v>
+      </c>
+    </row>
+    <row r="20" spans="1:16" ht="315" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="C20" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="B20" s="3" t="s">
-        <v>126</v>
-      </c>
-      <c r="C20" s="3" t="s">
-        <v>127</v>
-      </c>
       <c r="D20" s="3" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="E20" s="3" t="s">
         <v>37</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="H20" s="4"/>
       <c r="I20" s="4"/>
       <c r="J20" s="3" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="K20" s="3" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="L20" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M20" s="3" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="N20" s="4">
-        <v>0.10150000000000001</v>
+        <v>0.10100000000000001</v>
       </c>
       <c r="O20" s="4">
         <v>64</v>
       </c>
       <c r="P20" s="4">
-        <v>10.15</v>
-      </c>
-    </row>
-    <row r="21" spans="1:16" ht="330" x14ac:dyDescent="0.25">
+        <v>6.46</v>
+      </c>
+    </row>
+    <row r="21" spans="1:16" ht="165" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="C21" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F21" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="G21" s="3" t="s">
         <v>127</v>
-      </c>
-      <c r="D21" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="E21" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="F21" s="3" t="s">
-        <v>132</v>
-      </c>
-      <c r="G21" s="3" t="s">
-        <v>129</v>
       </c>
       <c r="H21" s="4"/>
       <c r="I21" s="4"/>
       <c r="J21" s="3" t="s">
-        <v>83</v>
+        <v>137</v>
       </c>
       <c r="K21" s="3" t="s">
-        <v>130</v>
+        <v>22</v>
       </c>
       <c r="L21" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M21" s="3" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="N21" s="4">
-        <v>0.10100000000000001</v>
+        <v>7.3999999999999996E-2</v>
       </c>
       <c r="O21" s="4">
-        <v>64</v>
+        <v>32</v>
       </c>
       <c r="P21" s="4">
-        <v>6.46</v>
-      </c>
-    </row>
-    <row r="22" spans="1:16" ht="165" x14ac:dyDescent="0.25">
+        <v>2.37</v>
+      </c>
+    </row>
+    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="C22" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="F22" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="G22" s="3" t="s">
         <v>113</v>
-      </c>
-      <c r="D22" s="3" t="s">
-        <v>138</v>
-      </c>
-      <c r="E22" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="F22" s="3" t="s">
-        <v>136</v>
-      </c>
-      <c r="G22" s="3" t="s">
-        <v>129</v>
       </c>
       <c r="H22" s="4"/>
       <c r="I22" s="4"/>
       <c r="J22" s="3" t="s">
-        <v>139</v>
+        <v>82</v>
       </c>
       <c r="K22" s="3" t="s">
-        <v>22</v>
+        <v>128</v>
       </c>
       <c r="L22" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M22" s="3" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="N22" s="4">
-        <v>7.3999999999999996E-2</v>
+        <v>2.4E-2</v>
       </c>
       <c r="O22" s="4">
-        <v>32</v>
+        <v>4</v>
       </c>
       <c r="P22" s="4">
-        <v>2.37</v>
-      </c>
-    </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
+        <v>0.24</v>
+      </c>
+    </row>
+    <row r="23" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>141</v>
+        <v>116</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>142</v>
-      </c>
-      <c r="C23" s="4"/>
-      <c r="D23" s="4"/>
+        <v>143</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>144</v>
+      </c>
       <c r="E23" s="3" t="s">
         <v>37</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>141</v>
+        <v>116</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="H23" s="4"/>
       <c r="I23" s="4"/>
       <c r="J23" s="3" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="K23" s="3" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="L23" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M23" s="3" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="N23" s="4">
-        <v>0.1</v>
+        <v>2.4E-2</v>
       </c>
       <c r="O23" s="4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P23" s="4">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="24" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+        <v>0.24</v>
+      </c>
+    </row>
+    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="E24" s="3" t="s">
         <v>37</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="G24" s="3" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="H24" s="4"/>
       <c r="I24" s="4"/>
       <c r="J24" s="3" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="K24" s="3" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="L24" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M24" s="3" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="N24" s="4">
-        <v>2.4E-2</v>
+        <v>0.1</v>
       </c>
       <c r="O24" s="4">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="P24" s="4">
-        <v>0.24</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="25" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
-        <v>118</v>
+        <v>150</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="E25" s="3" t="s">
         <v>37</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>118</v>
+        <v>150</v>
       </c>
       <c r="G25" s="3" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="H25" s="4"/>
       <c r="I25" s="4"/>
       <c r="J25" s="3" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="K25" s="3" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="L25" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M25" s="3" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="N25" s="4">
-        <v>2.4E-2</v>
+        <v>0.1</v>
       </c>
       <c r="O25" s="4">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="P25" s="4">
-        <v>0.24</v>
-      </c>
-    </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>152</v>
-      </c>
-      <c r="C26" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="D26" s="3" t="s">
-        <v>153</v>
-      </c>
+        <v>155</v>
+      </c>
+      <c r="C26" s="4"/>
+      <c r="D26" s="4"/>
       <c r="E26" s="3" t="s">
         <v>37</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="G26" s="3" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="H26" s="4"/>
       <c r="I26" s="4"/>
       <c r="J26" s="3" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="K26" s="3" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="L26" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M26" s="3" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="N26" s="4">
         <v>0.1</v>
@@ -2334,41 +2280,37 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="27" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>156</v>
-      </c>
-      <c r="C27" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="D27" s="3" t="s">
-        <v>157</v>
-      </c>
+        <v>158</v>
+      </c>
+      <c r="C27" s="4"/>
+      <c r="D27" s="4"/>
       <c r="E27" s="3" t="s">
         <v>37</v>
       </c>
       <c r="F27" s="3" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="G27" s="3" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="H27" s="4"/>
       <c r="I27" s="4"/>
       <c r="J27" s="3" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="K27" s="3" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="L27" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M27" s="3" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="N27" s="4">
         <v>0.1</v>
@@ -2380,41 +2322,41 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="28" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="E28" s="3" t="s">
         <v>37</v>
       </c>
       <c r="F28" s="3" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="G28" s="3" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="H28" s="4"/>
       <c r="I28" s="4"/>
       <c r="J28" s="3" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="K28" s="3" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="L28" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M28" s="3" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="N28" s="4">
         <v>0.1</v>
@@ -2428,150 +2370,138 @@
     </row>
     <row r="29" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>113</v>
+        <v>166</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>165</v>
-      </c>
-      <c r="E29" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="F29" s="3" t="s">
-        <v>163</v>
-      </c>
-      <c r="G29" s="3" t="s">
-        <v>115</v>
-      </c>
+        <v>167</v>
+      </c>
+      <c r="E29" s="4"/>
+      <c r="F29" s="4"/>
+      <c r="G29" s="4"/>
       <c r="H29" s="4"/>
       <c r="I29" s="4"/>
       <c r="J29" s="3" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="K29" s="3" t="s">
-        <v>130</v>
+        <v>168</v>
       </c>
       <c r="L29" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M29" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="N29" s="4">
+        <v>3.98</v>
+      </c>
+      <c r="O29" s="4">
+        <v>4</v>
+      </c>
+      <c r="P29" s="4">
+        <v>15.92</v>
+      </c>
+    </row>
+    <row r="30" spans="1:16" ht="60" x14ac:dyDescent="0.25">
+      <c r="A30" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="C30" s="3" t="s">
         <v>166</v>
       </c>
-      <c r="N29" s="4">
-        <v>0.1</v>
-      </c>
-      <c r="O29" s="4">
-        <v>1</v>
-      </c>
-      <c r="P29" s="4">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="30" spans="1:16" ht="30" x14ac:dyDescent="0.25">
-      <c r="A30" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="B30" s="3" t="s">
-        <v>168</v>
-      </c>
-      <c r="C30" s="4"/>
-      <c r="D30" s="4"/>
+      <c r="D30" s="3" t="s">
+        <v>170</v>
+      </c>
       <c r="E30" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="F30" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="G30" s="3" t="s">
-        <v>115</v>
-      </c>
+        <v>172</v>
+      </c>
+      <c r="F30" s="4"/>
+      <c r="G30" s="4"/>
       <c r="H30" s="4"/>
       <c r="I30" s="4"/>
       <c r="J30" s="3" t="s">
-        <v>83</v>
+        <v>173</v>
       </c>
       <c r="K30" s="3" t="s">
-        <v>130</v>
+        <v>174</v>
       </c>
       <c r="L30" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M30" s="3" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="N30" s="4">
-        <v>0.1</v>
+        <v>7.33</v>
       </c>
       <c r="O30" s="4">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="P30" s="4">
-        <v>0.1</v>
+        <v>58.64</v>
       </c>
     </row>
     <row r="31" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
-        <v>170</v>
+        <v>176</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>113</v>
+        <v>178</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="E31" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="F31" s="3" t="s">
-        <v>170</v>
-      </c>
-      <c r="G31" s="3" t="s">
-        <v>115</v>
-      </c>
+        <v>179</v>
+      </c>
+      <c r="E31" s="4"/>
+      <c r="F31" s="4"/>
+      <c r="G31" s="4"/>
       <c r="H31" s="4"/>
       <c r="I31" s="4"/>
       <c r="J31" s="3" t="s">
-        <v>83</v>
+        <v>180</v>
       </c>
       <c r="K31" s="3" t="s">
-        <v>130</v>
+        <v>181</v>
       </c>
       <c r="L31" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M31" s="3" t="s">
-        <v>173</v>
+        <v>182</v>
       </c>
       <c r="N31" s="4">
-        <v>0.1</v>
+        <v>11.24</v>
       </c>
       <c r="O31" s="4">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="P31" s="4">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="32" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+        <v>44.96</v>
+      </c>
+    </row>
+    <row r="32" spans="1:16" ht="60" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
-        <v>174</v>
+        <v>183</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>175</v>
+        <v>184</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>176</v>
+        <v>185</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>177</v>
+        <v>186</v>
       </c>
       <c r="E32" s="4"/>
       <c r="F32" s="4"/>
@@ -2579,81 +2509,79 @@
       <c r="H32" s="4"/>
       <c r="I32" s="4"/>
       <c r="J32" s="3" t="s">
-        <v>83</v>
+        <v>187</v>
       </c>
       <c r="K32" s="3" t="s">
-        <v>178</v>
+        <v>188</v>
       </c>
       <c r="L32" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M32" s="3" t="s">
-        <v>179</v>
+        <v>189</v>
       </c>
       <c r="N32" s="4">
-        <v>3.98</v>
+        <v>3.34</v>
       </c>
       <c r="O32" s="4">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="P32" s="4">
-        <v>15.92</v>
-      </c>
-    </row>
-    <row r="33" spans="1:16" ht="60" x14ac:dyDescent="0.25">
+        <v>3.34</v>
+      </c>
+    </row>
+    <row r="33" spans="1:16" ht="90" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
-        <v>180</v>
+        <v>190</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>181</v>
+        <v>191</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>176</v>
+        <v>166</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>180</v>
-      </c>
-      <c r="E33" s="3" t="s">
-        <v>182</v>
-      </c>
+        <v>192</v>
+      </c>
+      <c r="E33" s="4"/>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
       <c r="H33" s="4"/>
       <c r="I33" s="4"/>
       <c r="J33" s="3" t="s">
-        <v>183</v>
+        <v>193</v>
       </c>
       <c r="K33" s="3" t="s">
-        <v>184</v>
+        <v>194</v>
       </c>
       <c r="L33" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M33" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="N33" s="4">
+        <v>3.37</v>
+      </c>
+      <c r="O33" s="4">
+        <v>3</v>
+      </c>
+      <c r="P33" s="4">
+        <v>10.11</v>
+      </c>
+    </row>
+    <row r="34" spans="1:16" ht="60" x14ac:dyDescent="0.25">
+      <c r="A34" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>197</v>
+      </c>
+      <c r="C34" s="3" t="s">
         <v>185</v>
       </c>
-      <c r="N33" s="4">
-        <v>7.33</v>
-      </c>
-      <c r="O33" s="4">
-        <v>8</v>
-      </c>
-      <c r="P33" s="4">
-        <v>58.64</v>
-      </c>
-    </row>
-    <row r="34" spans="1:16" ht="30" x14ac:dyDescent="0.25">
-      <c r="A34" s="3" t="s">
-        <v>186</v>
-      </c>
-      <c r="B34" s="3" t="s">
-        <v>187</v>
-      </c>
-      <c r="C34" s="3" t="s">
-        <v>188</v>
-      </c>
       <c r="D34" s="3" t="s">
-        <v>189</v>
+        <v>198</v>
       </c>
       <c r="E34" s="4"/>
       <c r="F34" s="4"/>
@@ -2661,119 +2589,117 @@
       <c r="H34" s="4"/>
       <c r="I34" s="4"/>
       <c r="J34" s="3" t="s">
-        <v>190</v>
+        <v>199</v>
       </c>
       <c r="K34" s="3" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="L34" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M34" s="3" t="s">
-        <v>192</v>
+        <v>200</v>
       </c>
       <c r="N34" s="4">
-        <v>11.24</v>
+        <v>3.34</v>
       </c>
       <c r="O34" s="4">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="P34" s="4">
-        <v>44.96</v>
+        <v>3.34</v>
       </c>
     </row>
     <row r="35" spans="1:16" ht="75" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
-        <v>193</v>
+        <v>201</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>194</v>
-      </c>
-      <c r="C35" s="3" t="s">
-        <v>195</v>
-      </c>
-      <c r="D35" s="3" t="s">
-        <v>196</v>
-      </c>
+        <v>202</v>
+      </c>
+      <c r="C35" s="4"/>
+      <c r="D35" s="4"/>
       <c r="E35" s="4"/>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
       <c r="H35" s="4"/>
       <c r="I35" s="4"/>
       <c r="J35" s="3" t="s">
-        <v>197</v>
+        <v>203</v>
       </c>
       <c r="K35" s="3" t="s">
-        <v>198</v>
+        <v>204</v>
       </c>
       <c r="L35" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M35" s="3" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="N35" s="4">
-        <v>3.34</v>
+        <v>2.4300000000000002</v>
       </c>
       <c r="O35" s="4">
         <v>1</v>
       </c>
       <c r="P35" s="4">
-        <v>3.34</v>
-      </c>
-    </row>
-    <row r="36" spans="1:16" ht="90" x14ac:dyDescent="0.25">
+        <v>2.4300000000000002</v>
+      </c>
+    </row>
+    <row r="36" spans="1:16" ht="75" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>201</v>
+        <v>207</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>176</v>
+        <v>208</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="E36" s="4"/>
-      <c r="F36" s="4"/>
+      <c r="F36" s="3" t="s">
+        <v>206</v>
+      </c>
       <c r="G36" s="4"/>
       <c r="H36" s="4"/>
       <c r="I36" s="4"/>
       <c r="J36" s="3" t="s">
-        <v>203</v>
+        <v>209</v>
       </c>
       <c r="K36" s="3" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="L36" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M36" s="3" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="N36" s="4">
-        <v>3.37</v>
+        <v>3.64</v>
       </c>
       <c r="O36" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="P36" s="4">
-        <v>10.11</v>
-      </c>
-    </row>
-    <row r="37" spans="1:16" ht="60" x14ac:dyDescent="0.25">
+        <v>3.64</v>
+      </c>
+    </row>
+    <row r="37" spans="1:16" ht="90" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>195</v>
+        <v>208</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>208</v>
+        <v>213</v>
       </c>
       <c r="E37" s="4"/>
       <c r="F37" s="4"/>
@@ -2781,106 +2707,30 @@
       <c r="H37" s="4"/>
       <c r="I37" s="4"/>
       <c r="J37" s="3" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="K37" s="3" t="s">
-        <v>198</v>
+        <v>213</v>
       </c>
       <c r="L37" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M37" s="3" t="s">
-        <v>210</v>
+        <v>215</v>
       </c>
       <c r="N37" s="4">
-        <v>3.34</v>
+        <v>4.8499999999999996</v>
       </c>
       <c r="O37" s="4">
         <v>1</v>
       </c>
       <c r="P37" s="4">
-        <v>3.34</v>
-      </c>
-    </row>
-    <row r="38" spans="1:16" ht="75" x14ac:dyDescent="0.25">
-      <c r="A38" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="B38" s="3" t="s">
-        <v>212</v>
-      </c>
-      <c r="C38" s="3" t="s">
-        <v>195</v>
-      </c>
-      <c r="D38" s="3" t="s">
-        <v>213</v>
-      </c>
-      <c r="E38" s="4"/>
-      <c r="F38" s="4"/>
-      <c r="G38" s="4"/>
-      <c r="H38" s="4"/>
-      <c r="I38" s="4"/>
-      <c r="J38" s="3" t="s">
-        <v>214</v>
-      </c>
-      <c r="K38" s="3" t="s">
-        <v>215</v>
-      </c>
-      <c r="L38" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="M38" s="3" t="s">
-        <v>216</v>
-      </c>
-      <c r="N38" s="4">
-        <v>2.2200000000000002</v>
-      </c>
-      <c r="O38" s="4">
-        <v>1</v>
-      </c>
-      <c r="P38" s="4">
-        <v>2.2200000000000002</v>
-      </c>
-    </row>
-    <row r="39" spans="1:16" ht="105" x14ac:dyDescent="0.25">
-      <c r="A39" s="3" t="s">
-        <v>217</v>
-      </c>
-      <c r="B39" s="3" t="s">
-        <v>218</v>
-      </c>
-      <c r="C39" s="3" t="s">
-        <v>176</v>
-      </c>
-      <c r="D39" s="3" t="s">
-        <v>219</v>
-      </c>
-      <c r="E39" s="4"/>
-      <c r="F39" s="4"/>
-      <c r="G39" s="4"/>
-      <c r="H39" s="4"/>
-      <c r="I39" s="4"/>
-      <c r="J39" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="K39" s="3" t="s">
-        <v>221</v>
-      </c>
-      <c r="L39" s="3" t="s">
-        <v>222</v>
-      </c>
-      <c r="M39" s="3" t="s">
-        <v>223</v>
-      </c>
-      <c r="N39" s="4"/>
-      <c r="O39" s="4">
-        <v>1</v>
-      </c>
-      <c r="P39" s="4"/>
+        <v>4.8499999999999996</v>
+      </c>
     </row>
   </sheetData>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.30555555555555558" right="0.30555555555555558" top="0.30555555555555558" bottom="0.30555555555555558" header="0" footer="0"/>
-  <pageSetup paperSize="9" scale="17" orientation="landscape" horizontalDpi="4294967292" verticalDpi="1200" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="16" orientation="landscape" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>